<commit_message>
Update transportation management system
</commit_message>
<xml_diff>
--- a/backend/test_users_400.xlsx
+++ b/backend/test_users_400.xlsx
@@ -121,10 +121,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -156,10 +156,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G401"/>
+  <dimension ref="A1:G405"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -9622,9 +9622,89 @@
         <v>India</v>
       </c>
     </row>
+    <row r="402">
+      <c r="A402" t="str">
+        <v>6</v>
+      </c>
+      <c r="B402" t="str">
+        <v>RAHUL</v>
+      </c>
+      <c r="C402" t="str">
+        <v>Jaihindpuram</v>
+      </c>
+      <c r="D402" t="str">
+        <v>Madurai</v>
+      </c>
+      <c r="F402" t="str">
+        <v>Tamil Nadu</v>
+      </c>
+      <c r="G402" t="str">
+        <v>India</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="str">
+        <v>7</v>
+      </c>
+      <c r="B403" t="str">
+        <v>RAGUL KRISHNA</v>
+      </c>
+      <c r="C403" t="str">
+        <v>Jaihindpuram</v>
+      </c>
+      <c r="D403" t="str">
+        <v>Madurai</v>
+      </c>
+      <c r="F403" t="str">
+        <v>Tamil Nadu</v>
+      </c>
+      <c r="G403" t="str">
+        <v>India</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="str">
+        <v>8</v>
+      </c>
+      <c r="B404" t="str">
+        <v>NABILESH</v>
+      </c>
+      <c r="C404" t="str">
+        <v>Vandiyur</v>
+      </c>
+      <c r="D404" t="str">
+        <v>Madurai</v>
+      </c>
+      <c r="F404" t="str">
+        <v>Tamil Nadu</v>
+      </c>
+      <c r="G404" t="str">
+        <v>India</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="str">
+        <v>9</v>
+      </c>
+      <c r="B405" t="str">
+        <v>SABARI</v>
+      </c>
+      <c r="C405" t="str">
+        <v>PERIYAR</v>
+      </c>
+      <c r="D405" t="str">
+        <v>Madurai</v>
+      </c>
+      <c r="F405" t="str">
+        <v>Tamil Nadu</v>
+      </c>
+      <c r="G405" t="str">
+        <v>India</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G401"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G405"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update latest transportation management changes with automation
</commit_message>
<xml_diff>
--- a/backend/test_users_400.xlsx
+++ b/backend/test_users_400.xlsx
@@ -121,10 +121,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -156,10 +156,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G405"/>
+  <dimension ref="A1:G408"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -9702,9 +9702,69 @@
         <v>India</v>
       </c>
     </row>
+    <row r="406">
+      <c r="A406" t="str">
+        <v>T S</v>
+      </c>
+      <c r="B406" t="str">
+        <v>RAHUL</v>
+      </c>
+      <c r="C406" t="str">
+        <v>Jaihindpuram</v>
+      </c>
+      <c r="D406" t="str">
+        <v>Madurai</v>
+      </c>
+      <c r="F406" t="str">
+        <v>Tamil Nadu</v>
+      </c>
+      <c r="G406" t="str">
+        <v>India</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="str">
+        <v>M U</v>
+      </c>
+      <c r="B407" t="str">
+        <v>RESHMA SRI</v>
+      </c>
+      <c r="C407" t="str">
+        <v>Arappayalam</v>
+      </c>
+      <c r="D407" t="str">
+        <v>Madurai</v>
+      </c>
+      <c r="F407" t="str">
+        <v>Tamil Nadu</v>
+      </c>
+      <c r="G407" t="str">
+        <v>India</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="str">
+        <v>123</v>
+      </c>
+      <c r="B408" t="str">
+        <v>yoheswari</v>
+      </c>
+      <c r="C408" t="str">
+        <v>Jaihindpuram</v>
+      </c>
+      <c r="D408" t="str">
+        <v>Madurai</v>
+      </c>
+      <c r="F408" t="str">
+        <v>Tamil Nadu</v>
+      </c>
+      <c r="G408" t="str">
+        <v>India</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G405"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G408"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>